<commit_message>
Merge real product data — 22 Tribal Zone earrings + sample categories (34 total products)
</commit_message>
<xml_diff>
--- a/New Style Inventory.xlsx
+++ b/New Style Inventory.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -740,174 +740,780 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>TZ4361-008</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Gold Kundan Cluster Studs</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>GOLD</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" t="n">
         <v>126</v>
       </c>
-      <c r="E2" s="6" t="n">
+      <c r="E2" t="n">
         <v>399</v>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>8903827098644</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="n">
+      <c r="F2" t="n">
+        <v>8903827098644</v>
+      </c>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="6" t="inlineStr"/>
-      <c r="I2" s="6" t="inlineStr"/>
-      <c r="J2" s="6" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>TZ4357-12</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Crystal Drop Earrings</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>GOLD</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" t="n">
         <v>120</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" t="n">
         <v>599</v>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>8903827098323</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="n">
+      <c r="F3" t="n">
+        <v>8903827098323</v>
+      </c>
+      <c r="G3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="6" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>TZ4357-19</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>White Pearl Studs</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>WHITE</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" t="n">
         <v>120</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" t="n">
         <v>599</v>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>8903827098392</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="n">
+      <c r="F4" t="n">
+        <v>8903827098392</v>
+      </c>
+      <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="6" t="inlineStr"/>
-      <c r="I4" s="6" t="inlineStr"/>
-      <c r="J4" s="6" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TZ4357-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>120</v>
+      </c>
+      <c r="E5" t="n">
+        <v>599</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8903827098248</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TZ4357-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>125</v>
+      </c>
+      <c r="E6" t="n">
+        <v>599</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8903827098408</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TZ4357-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E7" t="n">
+        <v>599</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8903827098408</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TZ4357-10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>119</v>
+      </c>
+      <c r="E8" t="n">
+        <v>599</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8903827098309</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TZ4357-8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>114</v>
+      </c>
+      <c r="E9" t="n">
+        <v>599</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8903827098286</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TZ4357-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>136</v>
+      </c>
+      <c r="E10" t="n">
+        <v>599</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8903827098217</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TZ4357-17</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>119</v>
+      </c>
+      <c r="E11" t="n">
+        <v>599</v>
+      </c>
+      <c r="F11" t="n">
+        <v>8903827098378</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>TZ4383-1</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Antique Gold Jhumka</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>GOLD</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D12" t="n">
         <v>123</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E12" t="n">
         <v>699</v>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>8903827097913</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n">
+      <c r="F12" t="n">
+        <v>8903827097913</v>
+      </c>
+      <c r="G12" t="n">
         <v>4</v>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
-      <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TZ4383-2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>123</v>
+      </c>
+      <c r="E13" t="n">
+        <v>699</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8903827097913</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TZ4383-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>61</v>
+      </c>
+      <c r="E14" t="n">
+        <v>699</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8903827098002</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TZ4383-10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>50</v>
+      </c>
+      <c r="E15" t="n">
+        <v>699</v>
+      </c>
+      <c r="F15" t="n">
+        <v>8903727099818</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TZ4383-10-SLV</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E16" t="n">
+        <v>699</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8903727099818</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>TZ4383-5</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Kundan Drop Earring</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>GOLD</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D17" t="n">
         <v>192</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E17" t="n">
         <v>699</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>8903827097951</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="n">
+      <c r="F17" t="n">
+        <v>8903827097951</v>
+      </c>
+      <c r="G17" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TZ4383-6</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>233</v>
+      </c>
+      <c r="E18" t="n">
+        <v>599</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8903827097968</v>
+      </c>
+      <c r="G18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TZ4383-3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>209</v>
+      </c>
+      <c r="E19" t="n">
+        <v>699</v>
+      </c>
+      <c r="F19" t="n">
+        <v>8903827097937</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TZ4383-7</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>198</v>
+      </c>
+      <c r="E20" t="n">
+        <v>599</v>
+      </c>
+      <c r="F20" t="n">
+        <v>8903827097975</v>
+      </c>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TZSSE-123</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>123</v>
+      </c>
+      <c r="E21" t="n">
+        <v>899</v>
+      </c>
+      <c r="F21" t="n">
+        <v>8903827081059</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TZSSE-677G</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>216</v>
+      </c>
+      <c r="E22" t="n">
+        <v>499</v>
+      </c>
+      <c r="F22" t="n">
+        <v>8903827076413</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HCSSE-663</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>EARRING</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>60</v>
+      </c>
+      <c r="E23" t="n">
+        <v>399</v>
+      </c>
+      <c r="F23" t="n">
+        <v>8903827077489</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>